<commit_message>
cambios en generar excel para adquisiciones
</commit_message>
<xml_diff>
--- a/src/templates/solicitud.xlsx
+++ b/src/templates/solicitud.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="98">
   <si>
     <t>Universidad Privada del Valle</t>
   </si>
@@ -78,13 +78,22 @@
     <t>Unidad Solicitante:</t>
   </si>
   <si>
+    <t>{{UNIDAD_SOLICITANTE}}</t>
+  </si>
+  <si>
     <t>Nro. Solicitud a ser Registrado:</t>
   </si>
   <si>
     <t>Centro de Costo:</t>
   </si>
   <si>
+    <t>{{CENTRO_COSTO}}</t>
+  </si>
+  <si>
     <t>Responsable:</t>
+  </si>
+  <si>
+    <t>{{RESPONSABLE}}</t>
   </si>
   <si>
     <t>Nro. Codigo de Inversión (Activos)</t>
@@ -93,10 +102,19 @@
     <t>FECHA EMISION DEL PEDIDO</t>
   </si>
   <si>
+    <t>{{FECHA_DIA}}</t>
+  </si>
+  <si>
+    <t>{{FECHA_MES}}</t>
+  </si>
+  <si>
+    <t>{{FECHA_ANIO}}</t>
+  </si>
+  <si>
     <t>Este formulario responde al procedimiento de adquisiciones de bienes y servicios aprobado, su uso es obligatorio en la Univalle</t>
   </si>
   <si>
-    <t xml:space="preserve">(Obligatorio) </t>
+    <t>{{JUSTIFICACION}}{{MONTO_LETRAS}}</t>
   </si>
   <si>
     <t>Cantidad</t>
@@ -123,7 +141,16 @@
     <t>OBSERVACIONES</t>
   </si>
   <si>
+    <t xml:space="preserve"> NECESARIOS PARA SEMESTRE I/2025</t>
+  </si>
+  <si>
     <t>Son:</t>
+  </si>
+  <si>
+    <t>TREINTA Y OCHO MIL QUINIENTOS DIEZ  00/100 BOLIVIANOS</t>
+  </si>
+  <si>
+    <t>{{MONTO_TOTAL}}</t>
   </si>
   <si>
     <t>Monto TOTAL</t>
@@ -1028,7 +1055,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="122">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1070,7 +1097,7 @@
     </xf>
     <xf borderId="16" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="17" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -1078,7 +1105,7 @@
     <xf borderId="18" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="19" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="3" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="20" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="21" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1102,7 +1129,7 @@
     <xf borderId="31" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="32" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="30" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="30" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1173,7 +1200,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="14" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
@@ -1187,7 +1214,9 @@
     </xf>
     <xf borderId="55" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="56" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="57" fillId="3" fontId="18" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="57" fillId="3" fontId="18" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="58" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="59" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="60" fillId="2" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1244,6 +1273,15 @@
     <xf borderId="69" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf borderId="7" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf borderId="7" fillId="3" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf borderId="30" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="43" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -1259,6 +1297,10 @@
     <xf borderId="50" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="57" fillId="3" fontId="18" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="7" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1727,7 +1769,9 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="23"/>
-      <c r="D8" s="24"/>
+      <c r="D8" s="24" t="s">
+        <v>5</v>
+      </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
@@ -1738,7 +1782,7 @@
       <c r="L8" s="6"/>
       <c r="M8" s="7"/>
       <c r="N8" s="25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="26"/>
       <c r="P8" s="26"/>
@@ -1750,11 +1794,13 @@
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="22" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="23"/>
-      <c r="D9" s="28"/>
+      <c r="D9" s="28" t="s">
+        <v>8</v>
+      </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
@@ -1775,11 +1821,13 @@
     </row>
     <row r="10" ht="27.0" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="23"/>
-      <c r="D10" s="28"/>
+      <c r="D10" s="28" t="s">
+        <v>10</v>
+      </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -1800,7 +1848,7 @@
     </row>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="35" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B11" s="36"/>
       <c r="C11" s="37"/>
@@ -1825,15 +1873,21 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B12" s="42"/>
       <c r="C12" s="43"/>
-      <c r="D12" s="44"/>
+      <c r="D12" s="44" t="s">
+        <v>13</v>
+      </c>
       <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
+      <c r="F12" s="44" t="s">
+        <v>14</v>
+      </c>
       <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="H12" s="44" t="s">
+        <v>15</v>
+      </c>
       <c r="I12" s="43"/>
       <c r="J12" s="45"/>
       <c r="K12" s="42"/>
@@ -1873,7 +1927,7 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="53" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B14" s="54"/>
       <c r="C14" s="54"/>
@@ -1898,7 +1952,7 @@
     </row>
     <row r="15" ht="15.0" customHeight="1">
       <c r="A15" s="58" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="42"/>
@@ -1954,15 +2008,15 @@
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="65" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="66" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="66" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
@@ -1973,12 +2027,12 @@
       <c r="L19" s="11"/>
       <c r="M19" s="12"/>
       <c r="N19" s="67" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="O19" s="26"/>
       <c r="P19" s="68"/>
       <c r="Q19" s="67" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
@@ -2000,12 +2054,12 @@
       <c r="L20" s="63"/>
       <c r="M20" s="64"/>
       <c r="N20" s="70" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="O20" s="71"/>
       <c r="P20" s="72"/>
       <c r="Q20" s="70" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="R20" s="71"/>
       <c r="S20" s="71"/>
@@ -2175,12 +2229,14 @@
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="78" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="D28" s="12"/>
-      <c r="E28" s="79"/>
+      <c r="E28" s="79" t="s">
+        <v>26</v>
+      </c>
       <c r="F28" s="11"/>
       <c r="G28" s="11"/>
       <c r="H28" s="11"/>
@@ -2223,9 +2279,11 @@
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="82" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="83"/>
+        <v>27</v>
+      </c>
+      <c r="B30" s="83" t="s">
+        <v>28</v>
+      </c>
       <c r="C30" s="84"/>
       <c r="D30" s="84"/>
       <c r="E30" s="84"/>
@@ -2240,7 +2298,9 @@
       <c r="N30" s="84"/>
       <c r="O30" s="84"/>
       <c r="P30" s="85"/>
-      <c r="Q30" s="86"/>
+      <c r="Q30" s="86" t="s">
+        <v>29</v>
+      </c>
       <c r="R30" s="87"/>
       <c r="S30" s="87"/>
       <c r="T30" s="87"/>
@@ -2264,7 +2324,7 @@
       <c r="O31" s="49"/>
       <c r="P31" s="50"/>
       <c r="Q31" s="90" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="R31" s="91"/>
       <c r="S31" s="91"/>
@@ -2288,7 +2348,7 @@
       <c r="N32" s="11"/>
       <c r="O32" s="12"/>
       <c r="P32" s="95" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="Q32" s="26"/>
       <c r="R32" s="26"/>
@@ -2322,30 +2382,30 @@
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="99" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B35" s="87"/>
       <c r="C35" s="87"/>
       <c r="D35" s="100"/>
       <c r="E35" s="101" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F35" s="87"/>
       <c r="G35" s="87"/>
       <c r="H35" s="100"/>
       <c r="I35" s="101" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="J35" s="87"/>
       <c r="K35" s="87"/>
       <c r="L35" s="100"/>
       <c r="M35" s="101" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="N35" s="87"/>
       <c r="O35" s="100"/>
       <c r="P35" s="101" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="Q35" s="87"/>
       <c r="R35" s="87"/>
@@ -2355,19 +2415,19 @@
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="102" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B36" s="71"/>
       <c r="C36" s="71"/>
       <c r="D36" s="72"/>
       <c r="E36" s="103" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F36" s="71"/>
       <c r="G36" s="71"/>
       <c r="H36" s="72"/>
       <c r="I36" s="103" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="J36" s="71"/>
       <c r="K36" s="71"/>
@@ -2376,7 +2436,7 @@
       <c r="N36" s="71"/>
       <c r="O36" s="72"/>
       <c r="P36" s="103" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="Q36" s="71"/>
       <c r="R36" s="71"/>
@@ -2398,26 +2458,26 @@
       <c r="K37" s="6"/>
       <c r="L37" s="7"/>
       <c r="M37" s="105" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="N37" s="6"/>
       <c r="O37" s="6"/>
       <c r="P37" s="7"/>
       <c r="Q37" s="106" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="R37" s="7"/>
       <c r="S37" s="107" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="T37" s="108" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="U37" s="19"/>
     </row>
     <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="109" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B38" s="26"/>
       <c r="C38" s="26"/>
@@ -2442,7 +2502,7 @@
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="110" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -3692,8 +3752,8 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="23"/>
-      <c r="D8" s="24" t="s">
-        <v>36</v>
+      <c r="D8" s="111" t="s">
+        <v>45</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -3705,7 +3765,7 @@
       <c r="L8" s="6"/>
       <c r="M8" s="7"/>
       <c r="N8" s="25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="26"/>
       <c r="P8" s="26"/>
@@ -3717,11 +3777,11 @@
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="22" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="23"/>
-      <c r="D9" s="28"/>
+      <c r="D9" s="112"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
@@ -3742,12 +3802,12 @@
     </row>
     <row r="10" ht="27.0" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="23"/>
-      <c r="D10" s="28" t="s">
-        <v>37</v>
+      <c r="D10" s="112" t="s">
+        <v>46</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -3769,7 +3829,7 @@
     </row>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="35" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B11" s="36"/>
       <c r="C11" s="37"/>
@@ -3794,19 +3854,19 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B12" s="42"/>
       <c r="C12" s="43"/>
-      <c r="D12" s="44">
+      <c r="D12" s="113">
         <v>18.0</v>
       </c>
       <c r="E12" s="43"/>
-      <c r="F12" s="44">
+      <c r="F12" s="113">
         <v>10.0</v>
       </c>
       <c r="G12" s="43"/>
-      <c r="H12" s="44">
+      <c r="H12" s="113">
         <v>2023.0</v>
       </c>
       <c r="I12" s="43"/>
@@ -3848,7 +3908,7 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="53" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B14" s="54"/>
       <c r="C14" s="54"/>
@@ -3872,8 +3932,8 @@
       <c r="U14" s="57"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
-      <c r="A15" s="111" t="s">
-        <v>38</v>
+      <c r="A15" s="114" t="s">
+        <v>47</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="42"/>
@@ -3928,16 +3988,16 @@
       <c r="U18" s="64"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="112" t="s">
-        <v>12</v>
+      <c r="A19" s="115" t="s">
+        <v>18</v>
       </c>
       <c r="B19" s="12"/>
-      <c r="C19" s="113" t="s">
-        <v>13</v>
+      <c r="C19" s="116" t="s">
+        <v>19</v>
       </c>
       <c r="D19" s="12"/>
-      <c r="E19" s="113" t="s">
-        <v>14</v>
+      <c r="E19" s="116" t="s">
+        <v>20</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
@@ -3947,13 +4007,13 @@
       <c r="K19" s="11"/>
       <c r="L19" s="11"/>
       <c r="M19" s="12"/>
-      <c r="N19" s="114" t="s">
-        <v>15</v>
+      <c r="N19" s="117" t="s">
+        <v>21</v>
       </c>
       <c r="O19" s="26"/>
       <c r="P19" s="68"/>
-      <c r="Q19" s="114" t="s">
-        <v>16</v>
+      <c r="Q19" s="117" t="s">
+        <v>22</v>
       </c>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
@@ -3974,13 +4034,13 @@
       <c r="K20" s="63"/>
       <c r="L20" s="63"/>
       <c r="M20" s="64"/>
-      <c r="N20" s="115" t="s">
-        <v>17</v>
+      <c r="N20" s="118" t="s">
+        <v>23</v>
       </c>
       <c r="O20" s="71"/>
       <c r="P20" s="72"/>
-      <c r="Q20" s="115" t="s">
-        <v>18</v>
+      <c r="Q20" s="118" t="s">
+        <v>24</v>
       </c>
       <c r="R20" s="71"/>
       <c r="S20" s="71"/>
@@ -3993,11 +4053,11 @@
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="77" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
@@ -4027,11 +4087,11 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="77" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -4061,11 +4121,11 @@
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="77" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
@@ -4095,11 +4155,11 @@
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="77" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
@@ -4129,11 +4189,11 @@
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="77" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
@@ -4163,11 +4223,11 @@
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="74" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="77" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
@@ -4197,11 +4257,11 @@
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="74" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="77" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
@@ -4231,11 +4291,11 @@
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="77" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
@@ -4265,11 +4325,11 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="77" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
@@ -4299,11 +4359,11 @@
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D30" s="7"/>
       <c r="E30" s="77" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
@@ -4333,11 +4393,11 @@
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="75" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
@@ -4367,11 +4427,11 @@
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="77" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
@@ -4401,11 +4461,11 @@
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="77" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
@@ -4435,11 +4495,11 @@
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="74" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="77" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -4469,11 +4529,11 @@
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="77" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
@@ -4503,11 +4563,11 @@
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="77" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
@@ -4537,11 +4597,11 @@
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D37" s="7"/>
       <c r="E37" s="77" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
@@ -4571,11 +4631,11 @@
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="77" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
@@ -4605,11 +4665,11 @@
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D39" s="7"/>
       <c r="E39" s="77" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
@@ -4639,11 +4699,11 @@
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D40" s="7"/>
       <c r="E40" s="77" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
@@ -4673,11 +4733,11 @@
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="77" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
@@ -4707,11 +4767,11 @@
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="77" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
@@ -4741,11 +4801,11 @@
       </c>
       <c r="B43" s="7"/>
       <c r="C43" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="77" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
@@ -4775,11 +4835,11 @@
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D44" s="7"/>
       <c r="E44" s="77" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
@@ -4809,11 +4869,11 @@
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="74" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="D45" s="7"/>
       <c r="E45" s="77" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
@@ -4843,11 +4903,11 @@
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D46" s="7"/>
       <c r="E46" s="77" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
@@ -4877,11 +4937,11 @@
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="74" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D47" s="7"/>
       <c r="E47" s="77" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
@@ -4911,11 +4971,11 @@
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D48" s="7"/>
       <c r="E48" s="77" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
@@ -4945,11 +5005,11 @@
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D49" s="7"/>
       <c r="E49" s="77" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
@@ -4979,11 +5039,11 @@
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="77" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
@@ -5013,11 +5073,11 @@
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="77" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
@@ -5047,11 +5107,11 @@
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="77" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
@@ -5081,11 +5141,11 @@
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="77" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
@@ -5115,11 +5175,11 @@
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="77" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
@@ -5149,11 +5209,11 @@
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D55" s="7"/>
       <c r="E55" s="77" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
@@ -5183,11 +5243,11 @@
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D56" s="7"/>
       <c r="E56" s="77" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
@@ -5217,11 +5277,11 @@
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D57" s="7"/>
       <c r="E57" s="77" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
@@ -5251,11 +5311,11 @@
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D58" s="7"/>
       <c r="E58" s="77" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
@@ -5285,11 +5345,11 @@
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D59" s="7"/>
       <c r="E59" s="77" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
@@ -5319,11 +5379,11 @@
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D60" s="7"/>
       <c r="E60" s="77" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6"/>
@@ -5353,11 +5413,11 @@
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="77" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
@@ -5387,11 +5447,11 @@
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="74" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D62" s="7"/>
       <c r="E62" s="77" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
@@ -5417,13 +5477,13 @@
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="78" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
       <c r="D63" s="12"/>
-      <c r="E63" s="79" t="s">
-        <v>85</v>
+      <c r="E63" s="119" t="s">
+        <v>94</v>
       </c>
       <c r="F63" s="11"/>
       <c r="G63" s="11"/>
@@ -5467,10 +5527,10 @@
     </row>
     <row r="65" ht="14.25" customHeight="1">
       <c r="A65" s="82" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B65" s="83" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="C65" s="84"/>
       <c r="D65" s="84"/>
@@ -5486,7 +5546,7 @@
       <c r="N65" s="84"/>
       <c r="O65" s="84"/>
       <c r="P65" s="85"/>
-      <c r="Q65" s="86">
+      <c r="Q65" s="120">
         <f>+SUM(Q21:U57)</f>
         <v>16645</v>
       </c>
@@ -5513,7 +5573,7 @@
       <c r="O66" s="49"/>
       <c r="P66" s="50"/>
       <c r="Q66" s="90" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="R66" s="91"/>
       <c r="S66" s="91"/>
@@ -5537,7 +5597,7 @@
       <c r="N67" s="11"/>
       <c r="O67" s="12"/>
       <c r="P67" s="95" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="Q67" s="26"/>
       <c r="R67" s="26"/>
@@ -5571,30 +5631,30 @@
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="99" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B70" s="87"/>
       <c r="C70" s="87"/>
       <c r="D70" s="100"/>
       <c r="E70" s="101" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F70" s="87"/>
       <c r="G70" s="87"/>
       <c r="H70" s="100"/>
       <c r="I70" s="101" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="J70" s="87"/>
       <c r="K70" s="87"/>
       <c r="L70" s="100"/>
       <c r="M70" s="101" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="N70" s="87"/>
       <c r="O70" s="100"/>
       <c r="P70" s="101" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="Q70" s="87"/>
       <c r="R70" s="87"/>
@@ -5604,19 +5664,19 @@
     </row>
     <row r="71" ht="14.25" customHeight="1">
       <c r="A71" s="102" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B71" s="71"/>
       <c r="C71" s="71"/>
       <c r="D71" s="72"/>
       <c r="E71" s="103" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F71" s="71"/>
       <c r="G71" s="71"/>
       <c r="H71" s="72"/>
       <c r="I71" s="103" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="J71" s="71"/>
       <c r="K71" s="71"/>
@@ -5625,7 +5685,7 @@
       <c r="N71" s="71"/>
       <c r="O71" s="72"/>
       <c r="P71" s="103" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="Q71" s="71"/>
       <c r="R71" s="71"/>
@@ -5647,26 +5707,26 @@
       <c r="K72" s="6"/>
       <c r="L72" s="7"/>
       <c r="M72" s="105" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="N72" s="6"/>
       <c r="O72" s="6"/>
       <c r="P72" s="7"/>
       <c r="Q72" s="106" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="R72" s="7"/>
       <c r="S72" s="107" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="T72" s="108" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="U72" s="19"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="109" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B73" s="26"/>
       <c r="C73" s="26"/>
@@ -5691,7 +5751,7 @@
     </row>
     <row r="74" ht="14.25" customHeight="1">
       <c r="A74" s="110" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B74" s="91"/>
       <c r="C74" s="91"/>
@@ -7081,8 +7141,8 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="23"/>
-      <c r="D8" s="24" t="s">
-        <v>36</v>
+      <c r="D8" s="111" t="s">
+        <v>45</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -7094,7 +7154,7 @@
       <c r="L8" s="6"/>
       <c r="M8" s="7"/>
       <c r="N8" s="25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="26"/>
       <c r="P8" s="26"/>
@@ -7106,11 +7166,11 @@
     </row>
     <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="22" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="23"/>
-      <c r="D9" s="28"/>
+      <c r="D9" s="112"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
@@ -7131,12 +7191,12 @@
     </row>
     <row r="10" ht="27.0" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="23"/>
-      <c r="D10" s="28" t="s">
-        <v>37</v>
+      <c r="D10" s="112" t="s">
+        <v>46</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -7158,7 +7218,7 @@
     </row>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="35" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B11" s="36"/>
       <c r="C11" s="37"/>
@@ -7183,19 +7243,19 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B12" s="42"/>
       <c r="C12" s="43"/>
-      <c r="D12" s="44">
+      <c r="D12" s="113">
         <v>18.0</v>
       </c>
       <c r="E12" s="43"/>
-      <c r="F12" s="44">
+      <c r="F12" s="113">
         <v>10.0</v>
       </c>
       <c r="G12" s="43"/>
-      <c r="H12" s="44">
+      <c r="H12" s="113">
         <v>2023.0</v>
       </c>
       <c r="I12" s="43"/>
@@ -7237,7 +7297,7 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="53" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B14" s="54"/>
       <c r="C14" s="54"/>
@@ -7261,8 +7321,8 @@
       <c r="U14" s="57"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
-      <c r="A15" s="111" t="s">
-        <v>87</v>
+      <c r="A15" s="114" t="s">
+        <v>96</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="42"/>
@@ -7317,16 +7377,16 @@
       <c r="U18" s="64"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="112" t="s">
-        <v>12</v>
+      <c r="A19" s="115" t="s">
+        <v>18</v>
       </c>
       <c r="B19" s="12"/>
-      <c r="C19" s="113" t="s">
-        <v>13</v>
+      <c r="C19" s="116" t="s">
+        <v>19</v>
       </c>
       <c r="D19" s="12"/>
-      <c r="E19" s="113" t="s">
-        <v>14</v>
+      <c r="E19" s="116" t="s">
+        <v>20</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
@@ -7336,13 +7396,13 @@
       <c r="K19" s="11"/>
       <c r="L19" s="11"/>
       <c r="M19" s="12"/>
-      <c r="N19" s="114" t="s">
-        <v>15</v>
+      <c r="N19" s="117" t="s">
+        <v>21</v>
       </c>
       <c r="O19" s="26"/>
       <c r="P19" s="68"/>
-      <c r="Q19" s="114" t="s">
-        <v>16</v>
+      <c r="Q19" s="117" t="s">
+        <v>22</v>
       </c>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
@@ -7363,13 +7423,13 @@
       <c r="K20" s="63"/>
       <c r="L20" s="63"/>
       <c r="M20" s="64"/>
-      <c r="N20" s="115" t="s">
-        <v>17</v>
+      <c r="N20" s="118" t="s">
+        <v>23</v>
       </c>
       <c r="O20" s="71"/>
       <c r="P20" s="72"/>
-      <c r="Q20" s="115" t="s">
-        <v>18</v>
+      <c r="Q20" s="118" t="s">
+        <v>24</v>
       </c>
       <c r="R20" s="71"/>
       <c r="S20" s="71"/>
@@ -7795,7 +7855,7 @@
       <c r="B39" s="7"/>
       <c r="C39" s="74"/>
       <c r="D39" s="7"/>
-      <c r="E39" s="116"/>
+      <c r="E39" s="121"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
@@ -7887,7 +7947,7 @@
       <c r="B43" s="7"/>
       <c r="C43" s="74"/>
       <c r="D43" s="7"/>
-      <c r="E43" s="116"/>
+      <c r="E43" s="121"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
@@ -8025,7 +8085,7 @@
       <c r="B49" s="7"/>
       <c r="C49" s="74"/>
       <c r="D49" s="7"/>
-      <c r="E49" s="116"/>
+      <c r="E49" s="121"/>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
@@ -8117,7 +8177,7 @@
       <c r="B53" s="7"/>
       <c r="C53" s="74"/>
       <c r="D53" s="7"/>
-      <c r="E53" s="116"/>
+      <c r="E53" s="121"/>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -8301,7 +8361,7 @@
       <c r="B61" s="7"/>
       <c r="C61" s="74"/>
       <c r="D61" s="7"/>
-      <c r="E61" s="116"/>
+      <c r="E61" s="121"/>
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -8413,13 +8473,13 @@
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="78" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
       <c r="D66" s="12"/>
-      <c r="E66" s="79" t="s">
-        <v>85</v>
+      <c r="E66" s="119" t="s">
+        <v>94</v>
       </c>
       <c r="F66" s="11"/>
       <c r="G66" s="11"/>
@@ -8463,10 +8523,10 @@
     </row>
     <row r="68" ht="14.25" customHeight="1">
       <c r="A68" s="82" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B68" s="83" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C68" s="84"/>
       <c r="D68" s="84"/>
@@ -8482,7 +8542,7 @@
       <c r="N68" s="84"/>
       <c r="O68" s="84"/>
       <c r="P68" s="85"/>
-      <c r="Q68" s="86">
+      <c r="Q68" s="120">
         <f>+SUM(Q21:U63)</f>
         <v>0</v>
       </c>
@@ -8509,7 +8569,7 @@
       <c r="O69" s="49"/>
       <c r="P69" s="50"/>
       <c r="Q69" s="90" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="R69" s="91"/>
       <c r="S69" s="91"/>
@@ -8533,7 +8593,7 @@
       <c r="N70" s="11"/>
       <c r="O70" s="12"/>
       <c r="P70" s="95" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="Q70" s="26"/>
       <c r="R70" s="26"/>
@@ -8567,30 +8627,30 @@
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="99" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B73" s="87"/>
       <c r="C73" s="87"/>
       <c r="D73" s="100"/>
       <c r="E73" s="101" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F73" s="87"/>
       <c r="G73" s="87"/>
       <c r="H73" s="100"/>
       <c r="I73" s="101" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="J73" s="87"/>
       <c r="K73" s="87"/>
       <c r="L73" s="100"/>
       <c r="M73" s="101" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="N73" s="87"/>
       <c r="O73" s="100"/>
       <c r="P73" s="101" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="Q73" s="87"/>
       <c r="R73" s="87"/>
@@ -8600,19 +8660,19 @@
     </row>
     <row r="74" ht="14.25" customHeight="1">
       <c r="A74" s="102" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B74" s="71"/>
       <c r="C74" s="71"/>
       <c r="D74" s="72"/>
       <c r="E74" s="103" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F74" s="71"/>
       <c r="G74" s="71"/>
       <c r="H74" s="72"/>
       <c r="I74" s="103" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="J74" s="71"/>
       <c r="K74" s="71"/>
@@ -8621,7 +8681,7 @@
       <c r="N74" s="71"/>
       <c r="O74" s="72"/>
       <c r="P74" s="103" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="Q74" s="71"/>
       <c r="R74" s="71"/>
@@ -8643,26 +8703,26 @@
       <c r="K75" s="6"/>
       <c r="L75" s="7"/>
       <c r="M75" s="105" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="N75" s="6"/>
       <c r="O75" s="6"/>
       <c r="P75" s="7"/>
       <c r="Q75" s="106" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="R75" s="7"/>
       <c r="S75" s="107" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="T75" s="108" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="U75" s="19"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="109" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B76" s="26"/>
       <c r="C76" s="26"/>
@@ -8687,7 +8747,7 @@
     </row>
     <row r="77" ht="14.25" customHeight="1">
       <c r="A77" s="110" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B77" s="91"/>
       <c r="C77" s="91"/>

</xml_diff>